<commit_message>
Demo rerun: 150 steps, 0 failed, with losses, the 25-year dispatch and the team
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jKkuHBjiyJimAVAdehBdi
</commit_message>
<xml_diff>
--- a/demo/arkaja-seci-rtc-tm-v/models/TenderToBid_SECI-set_financial_model.xlsx
+++ b/demo/arkaja-seci-rtc-tm-v/models/TenderToBid_SECI-set_financial_model.xlsx
@@ -128,7 +128,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="367">
   <si>
     <t>SECI Round-the-Clock · bid financial model</t>
   </si>
@@ -253,7 +253,7 @@
     <t>Solar</t>
   </si>
   <si>
-    <t>CUF (AC) 25.0% · Capex 4 ₹ cr/MW · O&amp;M 4 ₹ lakh/MW/yr</t>
+    <t>CUF (AC) 25.0% · Capex per MWac 4 ₹ cr/MWac · O&amp;M per MWac 4 ₹ lakh/MWac/yr</t>
   </si>
   <si>
     <t>Biomass</t>
@@ -1033,25 +1033,40 @@
     <t>DC:AC ratio</t>
   </si>
   <si>
+    <t>MWp/MWac</t>
+  </si>
+  <si>
     <t>Annual degradation</t>
   </si>
   <si>
+    <t>Capex per MWac</t>
+  </si>
+  <si>
+    <t>₹ cr/MWac</t>
+  </si>
+  <si>
+    <t>O&amp;M per MWac</t>
+  </si>
+  <si>
+    <t>₹ lakh/MWac/yr</t>
+  </si>
+  <si>
+    <t>Availability</t>
+  </si>
+  <si>
+    <t>CUF (fuel-limited)</t>
+  </si>
+  <si>
+    <t>Minimum stable load</t>
+  </si>
+  <si>
+    <t>Ramp rate</t>
+  </si>
+  <si>
     <t>Capex</t>
   </si>
   <si>
     <t>O&amp;M</t>
-  </si>
-  <si>
-    <t>Availability</t>
-  </si>
-  <si>
-    <t>CUF (fuel-limited)</t>
-  </si>
-  <si>
-    <t>Minimum stable load</t>
-  </si>
-  <si>
-    <t>Ramp rate</t>
   </si>
   <si>
     <t>Fuel cost</t>
@@ -12160,7 +12175,7 @@
         <v>1.4</v>
       </c>
       <c r="D6" t="s">
-        <v>88</v>
+        <v>301</v>
       </c>
       <c r="E6" s="73" t="s">
         <v>104</v>
@@ -12171,7 +12186,7 @@
         <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C7" s="72">
         <v>0.005</v>
@@ -12188,13 +12203,13 @@
         <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C8" s="71">
         <v>4</v>
       </c>
       <c r="D8" t="s">
-        <v>112</v>
+        <v>304</v>
       </c>
       <c r="E8" s="73" t="s">
         <v>104</v>
@@ -12205,13 +12220,13 @@
         <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C9" s="71">
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>121</v>
+        <v>306</v>
       </c>
       <c r="E9" s="73" t="s">
         <v>104</v>
@@ -12239,7 +12254,7 @@
         <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C11" s="72">
         <v>0.9</v>
@@ -12256,7 +12271,7 @@
         <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C12" s="72">
         <v>0.8</v>
@@ -12273,7 +12288,7 @@
         <v>42</v>
       </c>
       <c r="B13" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="C13" s="72">
         <v>0.55</v>
@@ -12290,7 +12305,7 @@
         <v>42</v>
       </c>
       <c r="B14" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C14" s="72">
         <v>0.01</v>
@@ -12307,7 +12322,7 @@
         <v>42</v>
       </c>
       <c r="B15" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="C15" s="71">
         <v>7</v>
@@ -12324,7 +12339,7 @@
         <v>42</v>
       </c>
       <c r="B16" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="C16" s="71">
         <v>40</v>
@@ -12341,7 +12356,7 @@
         <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C17" s="71">
         <v>4.5</v>
@@ -12358,7 +12373,7 @@
         <v>42</v>
       </c>
       <c r="B18" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="C18" s="72">
         <v>0.05</v>
@@ -12392,10 +12407,10 @@
         <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="C20" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="D20" t="s">
         <v>8</v>
@@ -12409,7 +12424,7 @@
         <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C21" s="72">
         <v>0.87</v>
@@ -12426,7 +12441,7 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="C22" s="72">
         <v>0.05</v>
@@ -12443,7 +12458,7 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C23" s="72">
         <v>0.95</v>
@@ -12460,7 +12475,7 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="C24" s="72">
         <v>0.02</v>
@@ -12480,7 +12495,7 @@
         <v>144</v>
       </c>
       <c r="C25" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="D25" t="s">
         <v>8</v>
@@ -12494,7 +12509,7 @@
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="C26" s="71">
         <v>1.2</v>
@@ -12511,7 +12526,7 @@
         <v>28</v>
       </c>
       <c r="B27" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="C27" s="71">
         <v>1.2</v>
@@ -12664,7 +12679,7 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C36" s="72">
         <v>0.05</v>
@@ -12707,7 +12722,7 @@
         <v>8</v>
       </c>
       <c r="E38" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -12724,7 +12739,7 @@
         <v>8</v>
       </c>
       <c r="E39" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -12741,7 +12756,7 @@
         <v>83</v>
       </c>
       <c r="E40" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -12758,7 +12773,7 @@
         <v>155</v>
       </c>
       <c r="E41" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -12775,7 +12790,7 @@
         <v>83</v>
       </c>
       <c r="E42" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -12792,7 +12807,7 @@
         <v>170</v>
       </c>
       <c r="E43" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -12800,7 +12815,7 @@
         <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="C44" s="72">
         <v>0.1</v>
@@ -12809,15 +12824,15 @@
         <v>83</v>
       </c>
       <c r="E44" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="B45" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="C45" t="s">
         <v>136</v>
@@ -12847,13 +12862,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="66" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="66" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="B1" s="66" t="s">
         <v>292</v>
       </c>
       <c r="C1" s="66" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -12913,13 +12928,13 @@
     </row>
     <row r="8" spans="1:3" s="66" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="66" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="B8" s="66" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="C8" s="66" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -12968,13 +12983,13 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="B13" s="8">
         <v>13561.777072949393</v>
       </c>
       <c r="C13" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -12985,7 +13000,7 @@
         <v>9493.243951064575</v>
       </c>
       <c r="C14" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -13022,87 +13037,87 @@
         <v>74</v>
       </c>
       <c r="C1" s="66" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D1" s="66" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="E1" s="66" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="F1" s="66" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="G1" s="66" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="H1" s="66" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="I1" s="66" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="J1" s="66" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="K1" s="66" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="L1" s="66" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="M1" s="66" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="N1" s="66" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="O1" s="66" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="P1" s="66" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="Q1" s="66" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="R1" s="66" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="S1" s="66" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="T1" s="66" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="U1" s="66" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="V1" s="66" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="W1" s="66" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="X1" s="66" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="Y1" s="66" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="Z1" s="66" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="AA1" s="66" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="AB1" s="66" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
@@ -13971,7 +13986,7 @@
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="B15" t="s">
         <v>8</v>
@@ -14401,7 +14416,7 @@
     </row>
     <row r="20" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.25">
@@ -14513,87 +14528,87 @@
         <v>74</v>
       </c>
       <c r="C1" s="66" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D1" s="66" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="E1" s="66" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="F1" s="66" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="G1" s="66" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="H1" s="66" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="I1" s="66" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="J1" s="66" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="K1" s="66" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="L1" s="66" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="M1" s="66" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="N1" s="66" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="O1" s="66" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="P1" s="66" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="Q1" s="66" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="R1" s="66" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="S1" s="66" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="T1" s="66" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="U1" s="66" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="V1" s="66" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="W1" s="66" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="X1" s="66" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="Y1" s="66" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="Z1" s="66" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="AA1" s="66" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="AB1" s="66" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
@@ -15462,7 +15477,7 @@
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="B15" t="s">
         <v>8</v>
@@ -16587,7 +16602,7 @@
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B30" t="s">
         <v>8</v>
@@ -16759,7 +16774,7 @@
     </row>
     <row r="32" spans="1:28" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>8</v>
@@ -16931,7 +16946,7 @@
     </row>
     <row r="34" spans="1:28" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>8</v>
@@ -17100,7 +17115,7 @@
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B36" t="s">
         <v>8</v>
@@ -17582,7 +17597,7 @@
     </row>
     <row r="44" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
     </row>
     <row r="45" spans="1:28" s="66" customFormat="1" x14ac:dyDescent="0.25">
@@ -17596,84 +17611,84 @@
         <v>76</v>
       </c>
       <c r="D45" s="66" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="E45" s="66" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="F45" s="66" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="G45" s="66" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="H45" s="66" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="I45" s="66" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="J45" s="66" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="K45" s="66" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="L45" s="66" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="M45" s="66" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="N45" s="66" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="O45" s="66" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="P45" s="66" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="Q45" s="66" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="R45" s="66" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="S45" s="66" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="T45" s="66" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="U45" s="66" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="V45" s="66" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="W45" s="66" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="X45" s="66" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="Y45" s="66" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="Z45" s="66" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="AA45" s="66" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="AB45" s="66" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="46" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="B46" t="s">
         <v>86</v>
@@ -17759,7 +17774,7 @@
     </row>
     <row r="47" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B47" t="s">
         <v>86</v>

</xml_diff>